<commit_message>
FINAL v2 - all features merged
</commit_message>
<xml_diff>
--- a/public/inventory_bulk_upload_template.xlsx
+++ b/public/inventory_bulk_upload_template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,18 +45,38 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00137333"/>
+    </font>
+    <font>
+      <color rgb="00137333"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+    </font>
+    <font>
+      <color rgb="001F4E79"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00833C00"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -83,9 +103,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,7 +116,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -467,92 +494,92 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Brand</t>
+          <t>Brand *</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Device Model</t>
+          <t>Device Model *</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Sample / HW Type</t>
+          <t>Sample / HW Type *</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>HW Stage</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+          <t>IMEI1 *</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>IMEI2</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Serial Number</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>VC ID</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Storage / RAM Variant</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Assigned Date *</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Sample Received Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>VC ID</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IMEI1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>IMEI2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Storage / RAM Variant</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Warehouse / Location</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Inventory Holder</t>
+          <t>Warehouse / Location *</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Inventory Holder *</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Assigned Date</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -576,50 +603,54 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DVT</t>
+          <t>352000001234567</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>352000001234568</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SN001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2565243</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>8GB/128GB</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>15-Jan-25</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2565243</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>352000001234567</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>352000001234568</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Black</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>8GB/128GB</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>10-Jan-25</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>WH-A</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>John Smith</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
     </row>
@@ -641,54 +672,58 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EVT</t>
+          <t>352000009876543</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>352000009876544</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2565273</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>8GB/256GB</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>01-Feb-25</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2565273</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>352000009876543</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>352000009876544</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>8GB/256GB</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>28-Jan-25</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>WH-B</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Jane Doe</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Raj Kumar</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Priority sample</t>
+          <t>Priority</t>
         </is>
       </c>
     </row>
@@ -710,64 +745,61 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PVT</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+          <t>352000005551234</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SN003</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>6GB/128GB</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>10-Mar-25</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>3525282</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>352000005551234</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>6GB/128GB</t>
-        </is>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>05-Mar-25</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>WH-A</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Raj Kumar</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation sqref="A2:A5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Brand" error="Select: itel, Tecno, Infinix, Oraimo, Villaon" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Brand" error="Select: itel, Tecno, Infinix, Oraimo, Villaon" type="list">
       <formula1>"itel,Tecno,Infinix,Oraimo,Villaon,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid HW Type" error="Select: PR0 / PR0-1 / PR1 / PR1-1 / PR2 / PIR / MPR" type="list">
+    <dataValidation sqref="C2:C10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid HW Type" error="Select: PR0 / PR0-1 / PR1 / PR1-1 / PR2 / PIR / MPR" type="list">
       <formula1>"PR0,PR0-1,PR1,PR1-1,PR2,PIR,MPR"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"EVT,DVT,PVT,MP,Other"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid IMEI1" error="IMEI1 must be exactly 15 digits" type="textLength" operator="equal">
+    <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid IMEI1" error="IMEI1 must be exactly 15 digits" type="textLength" operator="equal">
       <formula1>15</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid IMEI2" error="IMEI2 must be 15 digits if provided" type="textLength" operator="equal">
+    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid IMEI2" error="IMEI2 must be 15 digits if provided" type="textLength" operator="equal">
       <formula1>15</formula1>
     </dataValidation>
   </dataValidations>
@@ -781,16 +813,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="88" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>TRANSSION — Device Sample Inventory Upload Template v2</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TRANSSION — Device Sample Inventory Upload Template v3</t>
         </is>
       </c>
     </row>
@@ -798,16 +830,16 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>MANDATORY FIELDS (must not be empty):</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>MANDATORY FIELDS (red header — must not be empty):</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Brand | Device Model | Sample/HW Type | HW Stage | IMEI1 | Color | Storage/RAM | Location | Inventory Holder</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Brand | Device Model | Sample/HW Type | IMEI1 | Assigned Date | Warehouse/Location | Inventory Holder</t>
         </is>
       </c>
     </row>
@@ -815,62 +847,103 @@
       <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>OPTIONAL FIELDS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>IMEI2 | Serial Number | VC ID | Color | Storage/RAM | Sample Received Date | Assigned To | Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>DROPDOWN FIELDS:</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Brand       — itel | Tecno | Infinix | Oraimo | Villaon | Other</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>HW Type     — PR0 | PR0-1 | PR1 | PR1-1 | PR2 | PIR | MPR</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>HW Stage    — EVT | DVT | PVT | MP | Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>VALIDATION RULES:</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>IMEI1/2     — Must be exactly 15 digits</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Date Format — DD-MMM-YY  e.g. 15-Jan-25 | 01-Feb-25 | 10-Mar-25</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>IMEI1       — Mandatory, exactly 15 digits</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>IMEI2       — Optional, must be 15 digits IF provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Date Format — DD-MMM-YY  e.g. 15-Jan-25 | 01-Feb-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>PERFORMANCE NOTE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>This template supports 3000+ rows. System validates ALL rows first (fast), then inserts in batches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Duplicate detection is done via a single bulk database read — no per-row queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Use the 'Benchmark Upload' tab for competitor/benchmark devices.</t>
         </is>
@@ -905,62 +978,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Competitor Brand</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Device Model</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="12" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>Received Date</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>Serial Number / IMEI</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>Storage / RAM</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>Warehouse / Location</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Custodian</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>Purpose / Test Type</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>

</xml_diff>